<commit_message>
Cambios periodos e ingresos
</commit_message>
<xml_diff>
--- a/documentosEjemplo/Reporte de empleados.xlsx
+++ b/documentosEjemplo/Reporte de empleados.xlsx
@@ -624,7 +624,7 @@
       <c r="I9" s="5" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">ACTIVO</t>
+            <t xml:space="preserve">INACTIVO</t>
           </r>
         </is>
       </c>
@@ -5177,7 +5177,7 @@
       <c r="B87" s="4" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">EVA CRISITNA SÁNCHEZ VELASCO</t>
+            <t xml:space="preserve">EVA CRISTINA SANCHEZ VELASCO</t>
           </r>
         </is>
       </c>
@@ -5185,28 +5185,28 @@
       <c r="D87" s="4" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">GESTOR DE CRÉDITO</t>
+            <t xml:space="preserve">ANALISTA DE MESA DE CONTROL</t>
           </r>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">CARTERA</t>
+            <t xml:space="preserve">MESA DE CONTROL</t>
           </r>
         </is>
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
           <r>
+            <t xml:space="preserve">NO</t>
+          </r>
+        </is>
+      </c>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
+          <r>
             <t xml:space="preserve">SI</t>
-          </r>
-        </is>
-      </c>
-      <c r="G87" s="5" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">NO</t>
           </r>
         </is>
       </c>
@@ -18879,7 +18879,7 @@
       <c r="F306" s="5" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">SI</t>
+            <t xml:space="preserve">NO</t>
           </r>
         </is>
       </c>
@@ -18894,7 +18894,7 @@
       <c r="I306" s="5" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">ACTIVO</t>
+            <t xml:space="preserve">INACTIVO</t>
           </r>
         </is>
       </c>
@@ -20599,7 +20599,7 @@
       <c r="F334" s="5" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">SI</t>
+            <t xml:space="preserve">NO</t>
           </r>
         </is>
       </c>
@@ -20614,7 +20614,7 @@
       <c r="I334" s="5" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">ACTIVO</t>
+            <t xml:space="preserve">INACTIVO</t>
           </r>
         </is>
       </c>
@@ -26983,7 +26983,7 @@
       <c r="F436" s="5" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">SI</t>
+            <t xml:space="preserve">NO</t>
           </r>
         </is>
       </c>
@@ -26998,7 +26998,7 @@
       <c r="I436" s="5" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">ACTIVO</t>
+            <t xml:space="preserve">INACTIVO</t>
           </r>
         </is>
       </c>
@@ -28919,7 +28919,7 @@
       <c r="F467" s="5" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">NO</t>
+            <t xml:space="preserve">SI</t>
           </r>
         </is>
       </c>
@@ -29019,7 +29019,7 @@
       <c r="B469" s="4" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">RODOLFO TONATIHU GUTIERREZ LEON Y VELEZ</t>
+            <t xml:space="preserve">RODOLFO TONATIUH GUTIERREZ LEON Y VELEZ</t>
           </r>
         </is>
       </c>
@@ -30331,7 +30331,7 @@
       <c r="F490" s="5" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">SI</t>
+            <t xml:space="preserve">NO</t>
           </r>
         </is>
       </c>
@@ -30346,7 +30346,7 @@
       <c r="I490" s="5" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">ACTIVO</t>
+            <t xml:space="preserve">INACTIVO</t>
           </r>
         </is>
       </c>
@@ -30357,32 +30357,410 @@
       <c r="L490" s="6" t="inlineStr"/>
     </row>
     <row r="491" customHeight="1" ht="10">
-      <c r="A491" s="2" t="inlineStr">
+      <c r="A491" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">ORI21932</t>
+          </r>
+        </is>
+      </c>
+      <c r="B491" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">ALBINO REYES VASQUEZ</t>
+          </r>
+        </is>
+      </c>
+      <c r="C491" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">2722141789</t>
+          </r>
+        </is>
+      </c>
+      <c r="D491" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">GESTOR DE CRÉDITO</t>
+          </r>
+        </is>
+      </c>
+      <c r="E491" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">Operativo</t>
+          </r>
+        </is>
+      </c>
+      <c r="F491" s="5" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">SI</t>
+          </r>
+        </is>
+      </c>
+      <c r="G491" s="5" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">NO</t>
+          </r>
+        </is>
+      </c>
+      <c r="H491" s="5" t="inlineStr"/>
+      <c r="I491" s="5" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">ACTIVO</t>
+          </r>
+        </is>
+      </c>
+      <c r="J491" s="6">
+        <v>46131.0</v>
+      </c>
+      <c r="K491" s="6" t="inlineStr"/>
+      <c r="L491" s="6" t="inlineStr"/>
+    </row>
+    <row r="492" customHeight="1" ht="10">
+      <c r="A492" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">CUE06937</t>
+          </r>
+        </is>
+      </c>
+      <c r="B492" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">YULIANA DIAZ RODRIGUEZ</t>
+          </r>
+        </is>
+      </c>
+      <c r="C492" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">7772278630</t>
+          </r>
+        </is>
+      </c>
+      <c r="D492" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">GERENTE</t>
+          </r>
+        </is>
+      </c>
+      <c r="E492" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">GERENCIAL</t>
+          </r>
+        </is>
+      </c>
+      <c r="F492" s="5" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">SI</t>
+          </r>
+        </is>
+      </c>
+      <c r="G492" s="5" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">NO</t>
+          </r>
+        </is>
+      </c>
+      <c r="H492" s="5" t="inlineStr"/>
+      <c r="I492" s="5" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">ACTIVO</t>
+          </r>
+        </is>
+      </c>
+      <c r="J492" s="6">
+        <v>46174.0</v>
+      </c>
+      <c r="K492" s="6" t="inlineStr"/>
+      <c r="L492" s="6" t="inlineStr"/>
+    </row>
+    <row r="493" customHeight="1" ht="10">
+      <c r="A493" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">CUE10938</t>
+          </r>
+        </is>
+      </c>
+      <c r="B493" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">JONATHAN DAVID ZARATE MIRANDA</t>
+          </r>
+        </is>
+      </c>
+      <c r="C493" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">7777115917</t>
+          </r>
+        </is>
+      </c>
+      <c r="D493" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">SUBGERENTE</t>
+          </r>
+        </is>
+      </c>
+      <c r="E493" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">GERENCIAL</t>
+          </r>
+        </is>
+      </c>
+      <c r="F493" s="5" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">SI</t>
+          </r>
+        </is>
+      </c>
+      <c r="G493" s="5" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">NO</t>
+          </r>
+        </is>
+      </c>
+      <c r="H493" s="5" t="inlineStr"/>
+      <c r="I493" s="5" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">ACTIVO</t>
+          </r>
+        </is>
+      </c>
+      <c r="J493" s="6">
+        <v>46174.0</v>
+      </c>
+      <c r="K493" s="6" t="inlineStr"/>
+      <c r="L493" s="6" t="inlineStr"/>
+    </row>
+    <row r="494" customHeight="1" ht="10">
+      <c r="A494" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">ORI11939</t>
+          </r>
+        </is>
+      </c>
+      <c r="B494" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">VACANTE JALAPILLA </t>
+          </r>
+        </is>
+      </c>
+      <c r="C494" s="4" t="inlineStr"/>
+      <c r="D494" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">GESTOR DE CRÉDITO</t>
+          </r>
+        </is>
+      </c>
+      <c r="E494" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">Operativo</t>
+          </r>
+        </is>
+      </c>
+      <c r="F494" s="5" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">NO</t>
+          </r>
+        </is>
+      </c>
+      <c r="G494" s="5" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">NO</t>
+          </r>
+        </is>
+      </c>
+      <c r="H494" s="5" t="inlineStr"/>
+      <c r="I494" s="5" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">INACTIVO</t>
+          </r>
+        </is>
+      </c>
+      <c r="J494" s="6">
+        <v>46174.0</v>
+      </c>
+      <c r="K494" s="6" t="inlineStr"/>
+      <c r="L494" s="6" t="inlineStr"/>
+    </row>
+    <row r="495" customHeight="1" ht="10">
+      <c r="A495" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">ORI20945</t>
+          </r>
+        </is>
+      </c>
+      <c r="B495" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">DAVID RUIZ SALGADO</t>
+          </r>
+        </is>
+      </c>
+      <c r="C495" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">2721525623</t>
+          </r>
+        </is>
+      </c>
+      <c r="D495" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">GESTOR DE CRÉDITO</t>
+          </r>
+        </is>
+      </c>
+      <c r="E495" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">Operativo</t>
+          </r>
+        </is>
+      </c>
+      <c r="F495" s="5" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">SI</t>
+          </r>
+        </is>
+      </c>
+      <c r="G495" s="5" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">NO</t>
+          </r>
+        </is>
+      </c>
+      <c r="H495" s="5" t="inlineStr"/>
+      <c r="I495" s="5" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">ACTIVO</t>
+          </r>
+        </is>
+      </c>
+      <c r="J495" s="6">
+        <v>46181.0</v>
+      </c>
+      <c r="K495" s="6" t="inlineStr"/>
+      <c r="L495" s="6" t="inlineStr"/>
+    </row>
+    <row r="496" customHeight="1" ht="10">
+      <c r="A496" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">CUE05946</t>
+          </r>
+        </is>
+      </c>
+      <c r="B496" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">VERONICA ELIZABETH LOZADA MONDRAGON</t>
+          </r>
+        </is>
+      </c>
+      <c r="C496" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">7772583560</t>
+          </r>
+        </is>
+      </c>
+      <c r="D496" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">GESTOR DE CRÉDITO</t>
+          </r>
+        </is>
+      </c>
+      <c r="E496" s="4" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">Operativo</t>
+          </r>
+        </is>
+      </c>
+      <c r="F496" s="5" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">SI</t>
+          </r>
+        </is>
+      </c>
+      <c r="G496" s="5" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">NO</t>
+          </r>
+        </is>
+      </c>
+      <c r="H496" s="5" t="inlineStr"/>
+      <c r="I496" s="5" t="inlineStr">
+        <is>
+          <r>
+            <t xml:space="preserve">ACTIVO</t>
+          </r>
+        </is>
+      </c>
+      <c r="J496" s="6">
+        <v>46182.0</v>
+      </c>
+      <c r="K496" s="6" t="inlineStr"/>
+      <c r="L496" s="6" t="inlineStr"/>
+    </row>
+    <row r="497" customHeight="1" ht="10">
+      <c r="A497" s="2" t="inlineStr">
         <is>
           <r>
             <t xml:space="preserve">LENDUS</t>
           </r>
         </is>
       </c>
-      <c r="B491" s="7">
-        <v>46169.386124571785</v>
-      </c>
-      <c r="C491" s="7" t="inlineStr"/>
-      <c r="D491" s="7" t="inlineStr"/>
-      <c r="E491" s="7" t="inlineStr"/>
-      <c r="F491" s="7" t="inlineStr"/>
-      <c r="G491" s="7" t="inlineStr"/>
-      <c r="H491" s="8" t="inlineStr">
+      <c r="B497" s="7">
+        <v>46187.84221871523</v>
+      </c>
+      <c r="C497" s="7" t="inlineStr"/>
+      <c r="D497" s="7" t="inlineStr"/>
+      <c r="E497" s="7" t="inlineStr"/>
+      <c r="F497" s="7" t="inlineStr"/>
+      <c r="G497" s="7" t="inlineStr"/>
+      <c r="H497" s="8" t="inlineStr">
         <is>
           <r>
             <t xml:space="preserve">Pagina 1 de</t>
           </r>
         </is>
       </c>
-      <c r="I491" s="8" t="inlineStr"/>
-      <c r="J491" s="8" t="inlineStr"/>
-      <c r="K491" s="9" t="inlineStr"/>
-      <c r="L491" s="10" t="inlineStr">
+      <c r="I497" s="8" t="inlineStr"/>
+      <c r="J497" s="8" t="inlineStr"/>
+      <c r="K497" s="9" t="inlineStr"/>
+      <c r="L497" s="10" t="inlineStr">
         <is>
           <r>
             <t xml:space="preserve"> 1</t>
@@ -31369,8 +31747,20 @@
     <mergeCell ref="J489:L489"/>
     <mergeCell ref="G490:H490"/>
     <mergeCell ref="J490:L490"/>
-    <mergeCell ref="B491:G491"/>
-    <mergeCell ref="H491:J491"/>
+    <mergeCell ref="G491:H491"/>
+    <mergeCell ref="J491:L491"/>
+    <mergeCell ref="G492:H492"/>
+    <mergeCell ref="J492:L492"/>
+    <mergeCell ref="G493:H493"/>
+    <mergeCell ref="J493:L493"/>
+    <mergeCell ref="G494:H494"/>
+    <mergeCell ref="J494:L494"/>
+    <mergeCell ref="G495:H495"/>
+    <mergeCell ref="J495:L495"/>
+    <mergeCell ref="G496:H496"/>
+    <mergeCell ref="J496:L496"/>
+    <mergeCell ref="B497:G497"/>
+    <mergeCell ref="H497:J497"/>
   </mergeCells>
   <pageMargins left="0.0" right="0.0" top="0.0" bottom="0.00" header="0.0" footer="0.0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>